<commit_message>
Use writexl to generate the test fixtures
Replace the bespoke minimal xlsx writer in data-raw/make_test_fixtures.R with
writexl::write_xlsx and regenerate the fixtures. They read back to identical
values (muni physical 9/13, budget 10/14, yishuv/sa attrs and column names all
unchanged), so the tests pass without modification. writexl stays a maintainer-
only tool (used in build-ignored data-raw, like readr), so it is not added to
DESCRIPTION. 84 tests, R CMD check --as-cran is 0 errors / 0 warnings / 0 notes.
</commit_message>
<xml_diff>
--- a/tests/testthat/fixtures/muni_2024_sample.xlsx
+++ b/tests/testthat/fixtures/muni_2024_sample.xlsx
@@ -1,1086 +1,1512 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
+  <bookViews>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+  </bookViews>
   <sheets>
     <sheet name="toc" sheetId="1" r:id="rId1"/>
     <sheet name="physical" sheetId="2" r:id="rId2"/>
     <sheet name="budget" sheetId="3" r:id="rId3"/>
   </sheets>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">toc</t>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>toc</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="B1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">רשויות מקומיות 2024</t>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>רשויות מקומיות 2024</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>x.1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>x.2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>x.3</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>x.4</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>x.5</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>x.6</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">כללי</t>
+          <t>כללי</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">שנת עדכון: 2024
+          <t>שנת עדכון: 2024_x000D_
 (אלא אם צוין אחרת)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2020</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024-25</t>
+          <t>2024-25</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">שם  הרשות</t>
+          <t>שם  הרשות</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">סמל הרשות</t>
+          <t>סמל הרשות</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">מחוז</t>
+          <t>מחוז</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">מעמד מוניציפלי</t>
+          <t>מעמד מוניציפלי</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">מרחק מגבול מחוז תל אביב (ק"מ)</t>
+          <t>מרחק מגבול מחוז תל אביב (ק"מ)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">שנת קבלת מעמד מוניציפלי</t>
+          <t>שנת קבלת מעמד מוניציפלי</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">מרחב ימי, רשויות מקומיות הגובלות בחוף הים</t>
+          <t>מרחב ימי, רשויות מקומיות הגובלות בחוף הים</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">מספר חברי מועצה</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
+          <t>מספר חברי מועצה</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">כלל ארצי</t>
+          <t>כלל ארצי</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">עיריות</t>
+          <t>עיריות</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">מועצות מקומיות</t>
+          <t>מועצות מקומיות</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">מועצות אזוריות</t>
+          <t>מועצות אזוריות</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">אום אל-פחם</t>
+          <t>אום אל-פחם</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2710</t>
+          <t>2710</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">חיפה</t>
+          <t>חיפה</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">60.581242748414603</t>
+          <t>60.581242748414603</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1984</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
+          <t>17</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">אופקים</t>
+          <t>אופקים</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">31</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">הדרום</t>
+          <t>הדרום</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">87.130838665736604</t>
+          <t>87.130838665736604</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1995</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">אור יהודה</t>
+          <t>אור יהודה</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">2400</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">תל אביב</t>
+          <t>תל אביב</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">1988</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">אור עקיבא</t>
+          <t>אור עקיבא</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">1020</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">חיפה</t>
+          <t>חיפה</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">39.407376186601297</t>
+          <t>39.407376186601297</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">2001</t>
+          <t>2001</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">13</t>
+          <t>13</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">אילת</t>
+          <t>אילת</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">2600</t>
+          <t>2600</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">הדרום</t>
+          <t>הדרום</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">323.002330261476</t>
+          <t>323.002330261476</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1959</t>
+          <t>1959</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
+          <t>17</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">אלעד</t>
+          <t>אלעד</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">1309</t>
+          <t>1309</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">המרכז</t>
+          <t>המרכז</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">11.5731964987549</t>
+          <t>11.5731964987549</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">2007</t>
+          <t>2007</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">אריאל</t>
+          <t>אריאל</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">3570</t>
+          <t>3570</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">אזור יהודה והשומרון</t>
+          <t>אזור יהודה והשומרון</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">33.278948675188197</t>
+          <t>33.278948675188197</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">1998</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve">13</t>
+          <t>13</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">אשדוד</t>
+          <t>אשדוד</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">70</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">הדרום</t>
+          <t>הדרום</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">28.488399573388499</t>
+          <t>28.488399573388499</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">1968</t>
+          <t>1968</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">29</t>
+          <t>29</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">אשקלון</t>
+          <t>אשקלון</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">7100</t>
+          <t>7100</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">הדרום</t>
+          <t>הדרום</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">43.6771470285587</t>
+          <t>43.6771470285587</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">1955</t>
+          <t>1955</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">25</t>
+          <t>25</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="B1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">נתונים כספיים של רשויות מקומיות לשנת 2024 (באלפי ש"ח)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>נתונים כספיים של רשויות מקומיות לשנת 2024 (באלפי ש"ח)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>x.1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>x.2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>x.3</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>x.4</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>x.5</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>x.6</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">כללי</t>
+          <t>כללי</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">תקבולים</t>
+          <t>תקבולים</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">שם הרשות</t>
+          <t>שם הרשות</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">סמל הרשות</t>
+          <t>סמל הרשות</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">מחוז</t>
+          <t>מחוז</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">מעמד מוניציפלי</t>
+          <t>מעמד מוניציפלי</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">סה"כ  אוכלוסייה בסוף השנה</t>
+          <t>סה"כ  אוכלוסייה בסוף השנה</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">אשכול
-מדד חברתי כלכלי 
+          <t>אשכול_x000D_
+מדד חברתי כלכלי _x000D_
 (משנת 2021, מ-1 עד 10, 1 הנמוך ביותר)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">סה"כ תקבולים (תקציב רגיל ותקציב בלתי רגיל)</t>
+          <t>סה"כ תקבולים (תקציב רגיל ותקציב בלתי רגיל)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">סה"כ הכנסות בתקציב הרגיל</t>
+          <t>סה"כ הכנסות בתקציב הרגיל</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">כלל ארצי</t>
+          <t>כלל ארצי</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">122659629.84232999</t>
+          <t>122659629.84232999</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">98698397.967330009</t>
+          <t>98698397.967330009</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">עיריות סך הכל</t>
+          <t>עיריות סך הכל</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7567443</t>
+          <t>7567443</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">93320847</t>
+          <t>93320847</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">74131187</t>
+          <t>74131187</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">מועצות מקומיות סך הכל</t>
+          <t>מועצות מקומיות סך הכל</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1375106</t>
+          <t>1375106</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">13677993.772359999</t>
+          <t>13677993.772359999</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">11507322.68736</t>
+          <t>11507322.68736</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">מועצות אזוריות סך הכל</t>
+          <t>מועצות אזוריות סך הכל</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1044343</t>
+          <t>1044343</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">15660789.069970001</t>
+          <t>15660789.069970001</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">13059888.279969998</t>
+          <t>13059888.279969998</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">אום אל-פחם</t>
+          <t>אום אל-פחם</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2710</t>
+          <t>2710</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">חיפה</t>
+          <t>חיפה</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">60209</t>
+          <t>60209</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">542734</t>
+          <t>542734</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">473292</t>
+          <t>473292</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">אופקים</t>
+          <t>אופקים</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">31</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">הדרום</t>
+          <t>הדרום</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">39893</t>
+          <t>39893</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">767791</t>
+          <t>767791</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">336435</t>
+          <t>336435</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">אור יהודה</t>
+          <t>אור יהודה</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">2400</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">תל אביב</t>
+          <t>תל אביב</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">41130</t>
+          <t>41130</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">741348</t>
+          <t>741348</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">479685</t>
+          <t>479685</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">אור עקיבא</t>
+          <t>אור עקיבא</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">1020</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">חיפה</t>
+          <t>חיפה</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">25922</t>
+          <t>25922</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">380062</t>
+          <t>380062</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">250622</t>
+          <t>250622</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">אילת</t>
+          <t>אילת</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">2600</t>
+          <t>2600</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">הדרום</t>
+          <t>הדרום</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">56004</t>
+          <t>56004</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">904236</t>
+          <t>904236</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">771666</t>
+          <t>771666</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">אלעד</t>
+          <t>אלעד</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1309</t>
+          <t>1309</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">המרכז</t>
+          <t>המרכז</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">50846</t>
+          <t>50846</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">348249</t>
+          <t>348249</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">295748</t>
+          <t>295748</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">אריאל</t>
+          <t>אריאל</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">3570</t>
+          <t>3570</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">אזור יהודה והשומרון</t>
+          <t>אזור יהודה והשומרון</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">22191</t>
+          <t>22191</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">237024</t>
+          <t>237024</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">182115</t>
+          <t>182115</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">אשדוד</t>
+          <t>אשדוד</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">70</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">הדרום</t>
+          <t>הדרום</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">228562</t>
+          <t>228562</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">2691942</t>
+          <t>2691942</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve">2346531</t>
+          <t>2346531</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">אשקלון</t>
+          <t>אשקלון</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">7100</t>
+          <t>7100</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">הדרום</t>
+          <t>הדרום</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">166864</t>
+          <t>166864</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">1773870</t>
+          <t>1773870</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">1553702</t>
+          <t>1553702</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">באקה אל-גרביה</t>
+          <t>באקה אל-גרביה</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">6000</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">חיפה</t>
+          <t>חיפה</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">עירייה</t>
+          <t>עירייה</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">31275</t>
+          <t>31275</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">251785</t>
+          <t>251785</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">226129</t>
+          <t>226129</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>